<commit_message>
Update links in Seguimiento-Clientes-Web to htmlpreview URLs
</commit_message>
<xml_diff>
--- a/Proyectos/Abril/Seguimiento-Clientes-Web.xlsx
+++ b/Proyectos/Abril/Seguimiento-Clientes-Web.xlsx
@@ -571,7 +571,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>https://allersec.github.io/Proyectos/Abril/16/ClinicaDentalCadillon/</t>
+          <t>https://htmlpreview.github.io/?https://github.com/AllerSec/Proyectos/blob/main/Proyectos/Abril/16/ClinicaDentalCadillon/index.html</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
@@ -623,7 +623,7 @@
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>https://allersec.github.io/Proyectos/Abril/16/ClinicaDentalElenaManterolaZabala/</t>
+          <t>https://htmlpreview.github.io/?https://github.com/AllerSec/Proyectos/blob/main/Proyectos/Abril/16/ClinicaDentalElenaManterolaZabala/index.html</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -675,7 +675,7 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>https://allersec.github.io/Proyectos/Abril/16/ClinicaDentalHaginlari/</t>
+          <t>https://htmlpreview.github.io/?https://github.com/AllerSec/Proyectos/blob/main/Proyectos/Abril/16/ClinicaDentalHaginlari/index.html</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
@@ -727,7 +727,7 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>https://allersec.github.io/Proyectos/Abril/16/MaiderZabalaFisioterapia/</t>
+          <t>https://htmlpreview.github.io/?https://github.com/AllerSec/Proyectos/blob/main/Proyectos/Abril/16/MaiderZabalaFisioterapia/index.html</t>
         </is>
       </c>
       <c r="I7" s="3" t="inlineStr">

</xml_diff>